<commit_message>
Docs: Updaten des Status der Risiken
</commit_message>
<xml_diff>
--- a/docs/Risikomanagement/RMMM-Liste.xlsx
+++ b/docs/Risikomanagement/RMMM-Liste.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30015"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30117"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8005F107-AC7E-4965-BEBD-4A3397B04A38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{713775FB-D3E0-42E6-A369-A2771142683D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="44">
   <si>
     <t>Risiko ID</t>
   </si>
@@ -105,6 +105,9 @@
     <t>Anstellung eines Testers</t>
   </si>
   <si>
+    <t>reduziert</t>
+  </si>
+  <si>
     <t>Frederik</t>
   </si>
   <si>
@@ -121,6 +124,9 @@
   </si>
   <si>
     <t>Begrenzte Anzahl an Rezepten in der Datenbank</t>
+  </si>
+  <si>
+    <t>eleminiert</t>
   </si>
   <si>
     <t>Eden</t>
@@ -637,6 +643,7 @@
     <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
     <col min="6" max="8" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="15.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="29.7109375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="14.28515625" bestFit="1" customWidth="1"/>
@@ -750,17 +757,17 @@
         <v>23</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K3" s="6">
         <v>46128</v>
       </c>
       <c r="M3" s="11"/>
       <c r="N3" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="60.75">
@@ -768,7 +775,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C4" s="4">
         <v>0.6</v>
@@ -781,26 +788,26 @@
         <v>2.4</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="K4" s="6">
         <v>46128</v>
       </c>
       <c r="M4" s="12"/>
       <c r="N4" s="13" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="121.5">
@@ -808,7 +815,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C5" s="4">
         <v>0.4</v>
@@ -821,19 +828,19 @@
         <v>2</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="K5" s="6">
         <v>46135</v>
@@ -844,7 +851,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C6" s="4">
         <v>0.6</v>
@@ -857,16 +864,16 @@
         <v>1.2</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J6" s="5" t="s">
         <v>18</v>

</xml_diff>